<commit_message>
Cap shift schedule at 6 working days in a row
Option B no longer ties offs to Mon-Sun weeks: each supervisor gets 2 days
off after every 3-6 working days (still 10 days off in the period), which
lets one supervisor cover each Sunday on rotation. The 6-day limit is now
checked up to Sun 1 Nov, and the solver runs single-threaded so rebuilds
give the same roster.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BfSP37ddbCt67XV4b3EwwG
</commit_message>
<xml_diff>
--- a/shift-schedule/Supervisor_Shift_Schedule_Sep-Oct_2026.xlsx
+++ b/shift-schedule/Supervisor_Shift_Schedule_Sep-Oct_2026.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -641,7 +641,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>1. T1, T2 and E each get 2 consecutive days off every week (Mon-Sun).</t>
+          <t>1. T1, T2 and E each get 2 consecutive days off a week (5 off blocks = 10 days in 28 Sep - 31 Oct).</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>6. Nobody works more than 7 days in a row; at least 3 working days between offs.</t>
+          <t>6. Nobody works more than 6 days in a row (checked up to Sun 1 Nov); at least 3 days between offs.</t>
         </is>
       </c>
     </row>
@@ -717,60 +717,67 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Off days move week to week. Everyone gets at least one Sunday off and one full Sat + Sun weekend off.</t>
+          <t>Offs are not tied to fixed weekdays: each person gets 2 days off after every 3-6 working days.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Tradeoff: with the rules above, only one person can cover every Sunday if that person never gets a</t>
+          <t>Exactly one supervisor covers each Sunday and the Sunday duty rotates between T1, T2 and E.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Sunday off (as in Option A). Sharing Sunday offs means some Sundays have 2-3 supervisors on duty.</t>
+          <t>Everyone gets at least one full Sat + Sun weekend off.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Note: if offs had to fall inside each Mon-Sun week with a 6-day limit, E would have to work every Sunday.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Why the tooling offs sit together</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>T1 and T2 switch shift after their offs, so to stay on opposite shifts their offs must be on the</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>T1 and T2 switch shift after their offs, so to stay on opposite shifts their offs must be on the</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>same days or directly one after the other.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Not considered</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Public holidays, leave, and the 24-27 Sep roster (keep the current one). Tell us to adjust.</t>
         </is>
@@ -2793,14 +2800,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
@@ -2810,12 +2817,12 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>T1, E</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
@@ -2838,14 +2845,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
@@ -2855,12 +2862,12 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>T1, E</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -2883,14 +2890,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
@@ -2900,12 +2907,12 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>T1, E</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -2928,29 +2935,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -2973,29 +2980,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
@@ -3018,29 +3025,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
           <t>E</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>T2</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -3063,9 +3070,9 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
@@ -3073,14 +3080,14 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
@@ -3108,29 +3115,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>M, E</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
@@ -3153,29 +3160,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, E</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
@@ -3198,29 +3205,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F18" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, E</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
@@ -3243,29 +3250,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, E</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
@@ -3288,29 +3295,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, E</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
@@ -3333,29 +3340,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E21" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
           <t>T1</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>E</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
@@ -3378,29 +3385,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="H22" s="17" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I22" s="17" t="inlineStr">
@@ -3423,14 +3430,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
@@ -3440,12 +3447,12 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
@@ -3468,14 +3475,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -3485,12 +3492,12 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
@@ -3513,14 +3520,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -3530,12 +3537,12 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
@@ -3558,14 +3565,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
@@ -3575,12 +3582,12 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
@@ -3603,14 +3610,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="F27" s="15" t="inlineStr">
@@ -3620,12 +3627,12 @@
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
@@ -3648,14 +3655,14 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
@@ -3665,12 +3672,12 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -3693,14 +3700,14 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
@@ -3710,12 +3717,12 @@
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>T2, E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I29" s="17" t="inlineStr">
@@ -3743,9 +3750,9 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
@@ -3755,7 +3762,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>M, T2, E</t>
+          <t>M, E</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -3788,9 +3795,9 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
@@ -3800,7 +3807,7 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>M, E</t>
+          <t>M, T2, E</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
@@ -3833,19 +3840,19 @@
           <t>2nd</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F32" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>M, E</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -3873,29 +3880,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>M, E</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
@@ -3918,29 +3925,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>M, E</t>
+          <t>M, T2</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1, E</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -3963,29 +3970,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F35" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1, E</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
@@ -4008,29 +4015,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
         </is>
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I36" s="17" t="inlineStr">
@@ -4053,9 +4060,9 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -4070,7 +4077,7 @@
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>M, T1</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
@@ -4103,14 +4110,14 @@
           <t>1st</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F38" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -4120,7 +4127,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -4143,29 +4150,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, T1</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -4188,29 +4195,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F40" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, T1, E</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
@@ -4233,29 +4240,29 @@
           <t>G</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E41" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F41" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>M, T2</t>
+          <t>M, T1, E</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>T1, E</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
@@ -4278,29 +4285,29 @@
           <t>OFF</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="F42" s="14" t="inlineStr">
-        <is>
-          <t>2nd</t>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>1st</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
+          <t>T1, E</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
           <t>T2</t>
-        </is>
-      </c>
-      <c r="H42" s="11" t="inlineStr">
-        <is>
-          <t>T1, E</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -4371,10 +4378,10 @@
         <v>10</v>
       </c>
       <c r="F46" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="11" t="n">
         <v>3</v>
-      </c>
-      <c r="G46" s="11" t="n">
-        <v>1</v>
       </c>
       <c r="H46" s="11" t="n">
         <v>1</v>
@@ -4388,19 +4395,19 @@
       </c>
       <c r="B47" s="9" t="n"/>
       <c r="C47" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D47" s="11" t="n">
         <v>11</v>
-      </c>
-      <c r="D47" s="11" t="n">
-        <v>13</v>
       </c>
       <c r="E47" s="11" t="n">
         <v>10</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H47" s="11" t="n">
         <v>1</v>
@@ -4414,19 +4421,19 @@
       </c>
       <c r="B48" s="9" t="n"/>
       <c r="C48" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="E48" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D48" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E48" s="11" t="n">
-        <v>8</v>
-      </c>
       <c r="F48" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G48" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H48" s="11" t="n">
         <v>1</v>

</xml_diff>